<commit_message>
add 13 new terms (JASPAR/JASIC/JSAE/SBOM/DCM/CCU/WPA/QNX/IPC/Auto-ISAC/J-Auto-ISAC/process-approval/etc) + TARA S/E/C detail
</commit_message>
<xml_diff>
--- a/docs/review-checklist.xlsx
+++ b/docs/review-checklist.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1218" uniqueCount="345">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1386" uniqueCount="393">
   <si>
     <t>No.</t>
   </si>
@@ -59,25 +59,49 @@
     <t>指摘事項・コメント</t>
   </si>
   <si>
+    <t>ccu</t>
+  </si>
+  <si>
+    <t>CCU</t>
+  </si>
+  <si>
+    <t>自動車部品</t>
+  </si>
+  <si>
+    <t>シーシーユー</t>
+  </si>
+  <si>
+    <t>Central/Connectivity Control Unit</t>
+  </si>
+  <si>
+    <t>2026-04-06</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
     <t>cv-joint</t>
   </si>
   <si>
     <t>CVジョイント</t>
   </si>
   <si>
-    <t>自動車部品</t>
-  </si>
-  <si>
     <t>シーブイジョイント</t>
   </si>
   <si>
     <t>Constant Velocity Joint</t>
   </si>
   <si>
-    <t>2026-04-06</t>
-  </si>
-  <si>
-    <t/>
+    <t>dcm</t>
+  </si>
+  <si>
+    <t>DCM</t>
+  </si>
+  <si>
+    <t>ディーシーエム</t>
+  </si>
+  <si>
+    <t>Data Communication Module</t>
   </si>
   <si>
     <t>ecu</t>
@@ -215,15 +239,27 @@
     <t>Three-Way Catalytic Converter</t>
   </si>
   <si>
+    <t>auto-isac</t>
+  </si>
+  <si>
+    <t>Auto-ISAC</t>
+  </si>
+  <si>
+    <t>サイバーセキュリティ</t>
+  </si>
+  <si>
+    <t>オートアイサック</t>
+  </si>
+  <si>
+    <t>Automotive Information Sharing and Analysis Center</t>
+  </si>
+  <si>
     <t>csms</t>
   </si>
   <si>
     <t>CSMS</t>
   </si>
   <si>
-    <t>サイバーセキュリティ</t>
-  </si>
-  <si>
     <t>シーエスエムエス</t>
   </si>
   <si>
@@ -266,6 +302,30 @@
     <t>ISO/SAE 21434 Road Vehicles - Cybersecurity Engineering</t>
   </si>
   <si>
+    <t>j-auto-isac</t>
+  </si>
+  <si>
+    <t>J-Auto-ISAC</t>
+  </si>
+  <si>
+    <t>ジェイオートアイサック</t>
+  </si>
+  <si>
+    <t>Japan Automotive ISAC</t>
+  </si>
+  <si>
+    <t>jasic</t>
+  </si>
+  <si>
+    <t>JASIC</t>
+  </si>
+  <si>
+    <t>ジャシック</t>
+  </si>
+  <si>
+    <t>Japan Automotive Security Information Center</t>
+  </si>
+  <si>
     <t>pki</t>
   </si>
   <si>
@@ -278,6 +338,18 @@
     <t>Public Key Infrastructure</t>
   </si>
   <si>
+    <t>sbom</t>
+  </si>
+  <si>
+    <t>SBOM</t>
+  </si>
+  <si>
+    <t>エスボム</t>
+  </si>
+  <si>
+    <t>Software Bill of Materials</t>
+  </si>
+  <si>
     <t>secoc</t>
   </si>
   <si>
@@ -326,6 +398,18 @@
     <t>VLAN Separation</t>
   </si>
   <si>
+    <t>wpa</t>
+  </si>
+  <si>
+    <t>WPA2/WPA3</t>
+  </si>
+  <si>
+    <t>ダブリューピーエーツースリー</t>
+  </si>
+  <si>
+    <t>Wi-Fi Protected Access 2/3</t>
+  </si>
+  <si>
     <t>secure-ota</t>
   </si>
   <si>
@@ -620,6 +704,18 @@
     <t>ISO 26262 Road Vehicles - Functional Safety</t>
   </si>
   <si>
+    <t>qnx</t>
+  </si>
+  <si>
+    <t>QNX</t>
+  </si>
+  <si>
+    <t>キューエヌエックス</t>
+  </si>
+  <si>
+    <t>QNX Neutrino RTOS</t>
+  </si>
+  <si>
     <t>severity</t>
   </si>
   <si>
@@ -662,6 +758,18 @@
     <t>Safety Goal</t>
   </si>
   <si>
+    <t>ipc</t>
+  </si>
+  <si>
+    <t>プロセス間通信（IPC）</t>
+  </si>
+  <si>
+    <t>プロセスカンツウシン</t>
+  </si>
+  <si>
+    <t>Inter-Process Communication</t>
+  </si>
+  <si>
     <t>freedom-from-interference</t>
   </si>
   <si>
@@ -902,6 +1010,30 @@
     <t>Global Technical Regulation</t>
   </si>
   <si>
+    <t>jaspar</t>
+  </si>
+  <si>
+    <t>JASPAR</t>
+  </si>
+  <si>
+    <t>ジャスパー</t>
+  </si>
+  <si>
+    <t>Japan Automotive Software Platform and Architecture</t>
+  </si>
+  <si>
+    <t>jsae</t>
+  </si>
+  <si>
+    <t>JSAE（自動車技術会）</t>
+  </si>
+  <si>
+    <t>ジェイサエ</t>
+  </si>
+  <si>
+    <t>Society of Automotive Engineers of Japan</t>
+  </si>
+  <si>
     <t>kvms</t>
   </si>
   <si>
@@ -1008,6 +1140,18 @@
   </si>
   <si>
     <t>World Forum for Harmonization of Vehicle Regulations</t>
+  </si>
+  <si>
+    <t>process-approval</t>
+  </si>
+  <si>
+    <t>プロセス認可</t>
+  </si>
+  <si>
+    <t>プロセスニンカ</t>
+  </si>
+  <si>
+    <t>Process Approval (A-SPICE Assessment)</t>
   </si>
   <si>
     <t>type-approval</t>
@@ -1464,7 +1608,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:O86"/>
+  <dimension ref="A1:O98"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -1684,10 +1828,10 @@
         <v>17</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="G5" s="6" t="s">
         <v>20</v>
@@ -1722,19 +1866,19 @@
         <v>5</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D6" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="G6" s="4" t="s">
         <v>20</v>
@@ -1769,19 +1913,19 @@
         <v>6</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="D7" s="6" t="s">
         <v>17</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="G7" s="6" t="s">
         <v>20</v>
@@ -1816,19 +1960,19 @@
         <v>7</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D8" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="G8" s="4" t="s">
         <v>20</v>
@@ -1863,19 +2007,19 @@
         <v>8</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D9" s="6" t="s">
         <v>17</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="F9" s="6" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="G9" s="6" t="s">
         <v>20</v>
@@ -1910,19 +2054,19 @@
         <v>9</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="D10" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="G10" s="4" t="s">
         <v>20</v>
@@ -1957,19 +2101,19 @@
         <v>10</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="D11" s="6" t="s">
         <v>17</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="F11" s="6" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="G11" s="6" t="s">
         <v>20</v>
@@ -2004,19 +2148,19 @@
         <v>11</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="D12" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="G12" s="4" t="s">
         <v>20</v>
@@ -2051,19 +2195,19 @@
         <v>12</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D13" s="6" t="s">
         <v>17</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="F13" s="6" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="G13" s="6" t="s">
         <v>20</v>
@@ -2098,19 +2242,19 @@
         <v>13</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="D14" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="G14" s="4" t="s">
         <v>20</v>
@@ -2145,19 +2289,19 @@
         <v>14</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="D15" s="6" t="s">
         <v>17</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="F15" s="6" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="G15" s="6" t="s">
         <v>20</v>
@@ -2192,19 +2336,19 @@
         <v>15</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="D16" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="G16" s="4" t="s">
         <v>20</v>
@@ -2239,19 +2383,19 @@
         <v>16</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D17" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="E17" s="6" t="s">
         <v>69</v>
       </c>
-      <c r="E17" s="6" t="s">
+      <c r="F17" s="6" t="s">
         <v>70</v>
-      </c>
-      <c r="F17" s="6" t="s">
-        <v>71</v>
       </c>
       <c r="G17" s="6" t="s">
         <v>20</v>
@@ -2286,19 +2430,19 @@
         <v>17</v>
       </c>
       <c r="B18" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="C18" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="C18" s="4" t="s">
+      <c r="D18" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E18" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="D18" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="E18" s="4" t="s">
+      <c r="F18" s="4" t="s">
         <v>74</v>
-      </c>
-      <c r="F18" s="4" t="s">
-        <v>75</v>
       </c>
       <c r="G18" s="4" t="s">
         <v>20</v>
@@ -2333,13 +2477,13 @@
         <v>18</v>
       </c>
       <c r="B19" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="C19" s="6" t="s">
         <v>76</v>
       </c>
-      <c r="C19" s="6" t="s">
+      <c r="D19" s="6" t="s">
         <v>77</v>
-      </c>
-      <c r="D19" s="6" t="s">
-        <v>69</v>
       </c>
       <c r="E19" s="6" t="s">
         <v>78</v>
@@ -2386,7 +2530,7 @@
         <v>81</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>69</v>
+        <v>77</v>
       </c>
       <c r="E20" s="4" t="s">
         <v>82</v>
@@ -2433,7 +2577,7 @@
         <v>85</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>69</v>
+        <v>77</v>
       </c>
       <c r="E21" s="6" t="s">
         <v>86</v>
@@ -2480,7 +2624,7 @@
         <v>89</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>69</v>
+        <v>77</v>
       </c>
       <c r="E22" s="4" t="s">
         <v>90</v>
@@ -2527,7 +2671,7 @@
         <v>93</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>69</v>
+        <v>77</v>
       </c>
       <c r="E23" s="6" t="s">
         <v>94</v>
@@ -2574,7 +2718,7 @@
         <v>97</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>69</v>
+        <v>77</v>
       </c>
       <c r="E24" s="4" t="s">
         <v>98</v>
@@ -2621,7 +2765,7 @@
         <v>101</v>
       </c>
       <c r="D25" s="6" t="s">
-        <v>69</v>
+        <v>77</v>
       </c>
       <c r="E25" s="6" t="s">
         <v>102</v>
@@ -2668,7 +2812,7 @@
         <v>105</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>69</v>
+        <v>77</v>
       </c>
       <c r="E26" s="4" t="s">
         <v>106</v>
@@ -2715,13 +2859,13 @@
         <v>109</v>
       </c>
       <c r="D27" s="6" t="s">
-        <v>69</v>
+        <v>77</v>
       </c>
       <c r="E27" s="6" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="F27" s="6" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="G27" s="6" t="s">
         <v>20</v>
@@ -2756,19 +2900,19 @@
         <v>27</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>69</v>
+        <v>77</v>
       </c>
       <c r="E28" s="4" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="F28" s="4" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="G28" s="4" t="s">
         <v>20</v>
@@ -2803,19 +2947,19 @@
         <v>28</v>
       </c>
       <c r="B29" s="6" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="C29" s="6" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="D29" s="6" t="s">
-        <v>69</v>
+        <v>77</v>
       </c>
       <c r="E29" s="6" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="F29" s="6" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="G29" s="6" t="s">
         <v>20</v>
@@ -2850,19 +2994,19 @@
         <v>29</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>69</v>
+        <v>77</v>
       </c>
       <c r="E30" s="4" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="F30" s="4" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="G30" s="4" t="s">
         <v>20</v>
@@ -2897,19 +3041,19 @@
         <v>30</v>
       </c>
       <c r="B31" s="6" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="C31" s="6" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="D31" s="6" t="s">
-        <v>123</v>
+        <v>77</v>
       </c>
       <c r="E31" s="6" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="F31" s="6" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="G31" s="6" t="s">
         <v>20</v>
@@ -2944,19 +3088,19 @@
         <v>31</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="D32" s="4" t="s">
-        <v>123</v>
+        <v>77</v>
       </c>
       <c r="E32" s="4" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="F32" s="4" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="G32" s="4" t="s">
         <v>20</v>
@@ -2991,19 +3135,19 @@
         <v>32</v>
       </c>
       <c r="B33" s="6" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C33" s="6" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="D33" s="6" t="s">
-        <v>123</v>
+        <v>77</v>
       </c>
       <c r="E33" s="6" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="F33" s="6" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="G33" s="6" t="s">
         <v>20</v>
@@ -3038,19 +3182,19 @@
         <v>33</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="D34" s="4" t="s">
-        <v>123</v>
+        <v>77</v>
       </c>
       <c r="E34" s="4" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F34" s="4" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="G34" s="4" t="s">
         <v>20</v>
@@ -3085,13 +3229,13 @@
         <v>34</v>
       </c>
       <c r="B35" s="6" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C35" s="6" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="D35" s="6" t="s">
-        <v>123</v>
+        <v>77</v>
       </c>
       <c r="E35" s="6" t="s">
         <v>140</v>
@@ -3138,13 +3282,13 @@
         <v>143</v>
       </c>
       <c r="D36" s="4" t="s">
-        <v>123</v>
+        <v>77</v>
       </c>
       <c r="E36" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="F36" s="4" t="s">
         <v>144</v>
-      </c>
-      <c r="F36" s="4" t="s">
-        <v>145</v>
       </c>
       <c r="G36" s="4" t="s">
         <v>20</v>
@@ -3179,19 +3323,19 @@
         <v>36</v>
       </c>
       <c r="B37" s="6" t="s">
+        <v>145</v>
+      </c>
+      <c r="C37" s="6" t="s">
         <v>146</v>
       </c>
-      <c r="C37" s="6" t="s">
+      <c r="D37" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="E37" s="6" t="s">
         <v>147</v>
       </c>
-      <c r="D37" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="E37" s="6" t="s">
+      <c r="F37" s="6" t="s">
         <v>148</v>
-      </c>
-      <c r="F37" s="6" t="s">
-        <v>149</v>
       </c>
       <c r="G37" s="6" t="s">
         <v>20</v>
@@ -3226,13 +3370,13 @@
         <v>37</v>
       </c>
       <c r="B38" s="4" t="s">
+        <v>149</v>
+      </c>
+      <c r="C38" s="4" t="s">
         <v>150</v>
       </c>
-      <c r="C38" s="4" t="s">
+      <c r="D38" s="4" t="s">
         <v>151</v>
-      </c>
-      <c r="D38" s="4" t="s">
-        <v>123</v>
       </c>
       <c r="E38" s="4" t="s">
         <v>152</v>
@@ -3279,7 +3423,7 @@
         <v>155</v>
       </c>
       <c r="D39" s="6" t="s">
-        <v>123</v>
+        <v>151</v>
       </c>
       <c r="E39" s="6" t="s">
         <v>156</v>
@@ -3326,7 +3470,7 @@
         <v>159</v>
       </c>
       <c r="D40" s="4" t="s">
-        <v>123</v>
+        <v>151</v>
       </c>
       <c r="E40" s="4" t="s">
         <v>160</v>
@@ -3373,7 +3517,7 @@
         <v>163</v>
       </c>
       <c r="D41" s="6" t="s">
-        <v>123</v>
+        <v>151</v>
       </c>
       <c r="E41" s="6" t="s">
         <v>164</v>
@@ -3420,13 +3564,13 @@
         <v>167</v>
       </c>
       <c r="D42" s="4" t="s">
-        <v>123</v>
+        <v>151</v>
       </c>
       <c r="E42" s="4" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="F42" s="4" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="G42" s="4" t="s">
         <v>20</v>
@@ -3461,13 +3605,13 @@
         <v>42</v>
       </c>
       <c r="B43" s="6" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="C43" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="D43" s="6" t="s">
-        <v>171</v>
+        <v>151</v>
       </c>
       <c r="E43" s="6" t="s">
         <v>172</v>
@@ -3514,7 +3658,7 @@
         <v>175</v>
       </c>
       <c r="D44" s="4" t="s">
-        <v>171</v>
+        <v>151</v>
       </c>
       <c r="E44" s="4" t="s">
         <v>176</v>
@@ -3561,7 +3705,7 @@
         <v>179</v>
       </c>
       <c r="D45" s="6" t="s">
-        <v>171</v>
+        <v>151</v>
       </c>
       <c r="E45" s="6" t="s">
         <v>180</v>
@@ -3608,7 +3752,7 @@
         <v>183</v>
       </c>
       <c r="D46" s="4" t="s">
-        <v>171</v>
+        <v>151</v>
       </c>
       <c r="E46" s="4" t="s">
         <v>184</v>
@@ -3655,7 +3799,7 @@
         <v>187</v>
       </c>
       <c r="D47" s="6" t="s">
-        <v>171</v>
+        <v>151</v>
       </c>
       <c r="E47" s="6" t="s">
         <v>188</v>
@@ -3702,7 +3846,7 @@
         <v>191</v>
       </c>
       <c r="D48" s="4" t="s">
-        <v>171</v>
+        <v>151</v>
       </c>
       <c r="E48" s="4" t="s">
         <v>192</v>
@@ -3749,13 +3893,13 @@
         <v>195</v>
       </c>
       <c r="D49" s="6" t="s">
-        <v>171</v>
+        <v>151</v>
       </c>
       <c r="E49" s="6" t="s">
+        <v>195</v>
+      </c>
+      <c r="F49" s="6" t="s">
         <v>196</v>
-      </c>
-      <c r="F49" s="6" t="s">
-        <v>197</v>
       </c>
       <c r="G49" s="6" t="s">
         <v>20</v>
@@ -3790,13 +3934,13 @@
         <v>49</v>
       </c>
       <c r="B50" s="4" t="s">
+        <v>197</v>
+      </c>
+      <c r="C50" s="4" t="s">
         <v>198</v>
       </c>
-      <c r="C50" s="4" t="s">
+      <c r="D50" s="4" t="s">
         <v>199</v>
-      </c>
-      <c r="D50" s="4" t="s">
-        <v>171</v>
       </c>
       <c r="E50" s="4" t="s">
         <v>200</v>
@@ -3843,7 +3987,7 @@
         <v>203</v>
       </c>
       <c r="D51" s="6" t="s">
-        <v>171</v>
+        <v>199</v>
       </c>
       <c r="E51" s="6" t="s">
         <v>204</v>
@@ -3890,7 +4034,7 @@
         <v>207</v>
       </c>
       <c r="D52" s="4" t="s">
-        <v>171</v>
+        <v>199</v>
       </c>
       <c r="E52" s="4" t="s">
         <v>208</v>
@@ -3937,13 +4081,13 @@
         <v>211</v>
       </c>
       <c r="D53" s="6" t="s">
-        <v>171</v>
+        <v>199</v>
       </c>
       <c r="E53" s="6" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="F53" s="6" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="G53" s="6" t="s">
         <v>20</v>
@@ -3978,19 +4122,19 @@
         <v>53</v>
       </c>
       <c r="B54" s="4" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="C54" s="4" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="D54" s="4" t="s">
-        <v>171</v>
+        <v>199</v>
       </c>
       <c r="E54" s="4" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="F54" s="4" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="G54" s="4" t="s">
         <v>20</v>
@@ -4025,19 +4169,19 @@
         <v>54</v>
       </c>
       <c r="B55" s="6" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="C55" s="6" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="D55" s="6" t="s">
-        <v>171</v>
+        <v>199</v>
       </c>
       <c r="E55" s="6" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="F55" s="6" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="G55" s="6" t="s">
         <v>20</v>
@@ -4072,19 +4216,19 @@
         <v>55</v>
       </c>
       <c r="B56" s="4" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="C56" s="4" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="D56" s="4" t="s">
-        <v>222</v>
+        <v>199</v>
       </c>
       <c r="E56" s="4" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="F56" s="4" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="G56" s="4" t="s">
         <v>20</v>
@@ -4119,19 +4263,19 @@
         <v>56</v>
       </c>
       <c r="B57" s="6" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="C57" s="6" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="D57" s="6" t="s">
-        <v>222</v>
+        <v>199</v>
       </c>
       <c r="E57" s="6" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="F57" s="6" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="G57" s="6" t="s">
         <v>20</v>
@@ -4166,19 +4310,19 @@
         <v>57</v>
       </c>
       <c r="B58" s="4" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="C58" s="4" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="D58" s="4" t="s">
-        <v>222</v>
+        <v>199</v>
       </c>
       <c r="E58" s="4" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="F58" s="4" t="s">
-        <v>230</v>
+        <v>233</v>
       </c>
       <c r="G58" s="4" t="s">
         <v>20</v>
@@ -4213,19 +4357,19 @@
         <v>58</v>
       </c>
       <c r="B59" s="6" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
       <c r="C59" s="6" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
       <c r="D59" s="6" t="s">
-        <v>233</v>
+        <v>199</v>
       </c>
       <c r="E59" s="6" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="F59" s="6" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="G59" s="6" t="s">
         <v>20</v>
@@ -4260,19 +4404,19 @@
         <v>59</v>
       </c>
       <c r="B60" s="4" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="C60" s="4" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="D60" s="4" t="s">
-        <v>233</v>
+        <v>199</v>
       </c>
       <c r="E60" s="4" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="F60" s="4" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="G60" s="4" t="s">
         <v>20</v>
@@ -4307,19 +4451,19 @@
         <v>60</v>
       </c>
       <c r="B61" s="6" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="C61" s="6" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="D61" s="6" t="s">
-        <v>233</v>
+        <v>199</v>
       </c>
       <c r="E61" s="6" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="F61" s="6" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="G61" s="6" t="s">
         <v>20</v>
@@ -4354,13 +4498,13 @@
         <v>61</v>
       </c>
       <c r="B62" s="4" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="C62" s="4" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="D62" s="4" t="s">
-        <v>233</v>
+        <v>199</v>
       </c>
       <c r="E62" s="4" t="s">
         <v>246</v>
@@ -4407,7 +4551,7 @@
         <v>249</v>
       </c>
       <c r="D63" s="6" t="s">
-        <v>233</v>
+        <v>199</v>
       </c>
       <c r="E63" s="6" t="s">
         <v>250</v>
@@ -4454,7 +4598,7 @@
         <v>253</v>
       </c>
       <c r="D64" s="4" t="s">
-        <v>233</v>
+        <v>199</v>
       </c>
       <c r="E64" s="4" t="s">
         <v>254</v>
@@ -4501,13 +4645,13 @@
         <v>257</v>
       </c>
       <c r="D65" s="6" t="s">
-        <v>233</v>
+        <v>258</v>
       </c>
       <c r="E65" s="6" t="s">
         <v>257</v>
       </c>
       <c r="F65" s="6" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="G65" s="6" t="s">
         <v>20</v>
@@ -4542,19 +4686,19 @@
         <v>65</v>
       </c>
       <c r="B66" s="4" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="C66" s="4" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="D66" s="4" t="s">
-        <v>233</v>
+        <v>258</v>
       </c>
       <c r="E66" s="4" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="F66" s="4" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="G66" s="4" t="s">
         <v>20</v>
@@ -4589,19 +4733,19 @@
         <v>66</v>
       </c>
       <c r="B67" s="6" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="C67" s="6" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="D67" s="6" t="s">
-        <v>233</v>
+        <v>258</v>
       </c>
       <c r="E67" s="6" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="F67" s="6" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="G67" s="6" t="s">
         <v>20</v>
@@ -4636,19 +4780,19 @@
         <v>67</v>
       </c>
       <c r="B68" s="4" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="C68" s="4" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="D68" s="4" t="s">
-        <v>233</v>
+        <v>269</v>
       </c>
       <c r="E68" s="4" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
       <c r="F68" s="4" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
       <c r="G68" s="4" t="s">
         <v>20</v>
@@ -4683,19 +4827,19 @@
         <v>68</v>
       </c>
       <c r="B69" s="6" t="s">
-        <v>268</v>
+        <v>272</v>
       </c>
       <c r="C69" s="6" t="s">
+        <v>273</v>
+      </c>
+      <c r="D69" s="6" t="s">
         <v>269</v>
       </c>
-      <c r="D69" s="6" t="s">
-        <v>233</v>
-      </c>
       <c r="E69" s="6" t="s">
-        <v>269</v>
+        <v>274</v>
       </c>
       <c r="F69" s="6" t="s">
-        <v>270</v>
+        <v>275</v>
       </c>
       <c r="G69" s="6" t="s">
         <v>20</v>
@@ -4730,19 +4874,19 @@
         <v>69</v>
       </c>
       <c r="B70" s="4" t="s">
-        <v>271</v>
+        <v>276</v>
       </c>
       <c r="C70" s="4" t="s">
-        <v>272</v>
+        <v>277</v>
       </c>
       <c r="D70" s="4" t="s">
-        <v>233</v>
+        <v>269</v>
       </c>
       <c r="E70" s="4" t="s">
-        <v>273</v>
+        <v>278</v>
       </c>
       <c r="F70" s="4" t="s">
-        <v>274</v>
+        <v>279</v>
       </c>
       <c r="G70" s="4" t="s">
         <v>20</v>
@@ -4777,19 +4921,19 @@
         <v>70</v>
       </c>
       <c r="B71" s="6" t="s">
-        <v>275</v>
+        <v>280</v>
       </c>
       <c r="C71" s="6" t="s">
-        <v>276</v>
+        <v>281</v>
       </c>
       <c r="D71" s="6" t="s">
-        <v>233</v>
+        <v>269</v>
       </c>
       <c r="E71" s="6" t="s">
-        <v>277</v>
+        <v>282</v>
       </c>
       <c r="F71" s="6" t="s">
-        <v>278</v>
+        <v>283</v>
       </c>
       <c r="G71" s="6" t="s">
         <v>20</v>
@@ -4824,19 +4968,19 @@
         <v>71</v>
       </c>
       <c r="B72" s="4" t="s">
-        <v>279</v>
+        <v>284</v>
       </c>
       <c r="C72" s="4" t="s">
-        <v>280</v>
+        <v>285</v>
       </c>
       <c r="D72" s="4" t="s">
-        <v>233</v>
+        <v>269</v>
       </c>
       <c r="E72" s="4" t="s">
-        <v>281</v>
+        <v>286</v>
       </c>
       <c r="F72" s="4" t="s">
-        <v>282</v>
+        <v>287</v>
       </c>
       <c r="G72" s="4" t="s">
         <v>20</v>
@@ -4871,19 +5015,19 @@
         <v>72</v>
       </c>
       <c r="B73" s="6" t="s">
-        <v>283</v>
+        <v>288</v>
       </c>
       <c r="C73" s="6" t="s">
-        <v>284</v>
+        <v>289</v>
       </c>
       <c r="D73" s="6" t="s">
-        <v>285</v>
+        <v>269</v>
       </c>
       <c r="E73" s="6" t="s">
-        <v>286</v>
+        <v>290</v>
       </c>
       <c r="F73" s="6" t="s">
-        <v>287</v>
+        <v>291</v>
       </c>
       <c r="G73" s="6" t="s">
         <v>20</v>
@@ -4918,19 +5062,19 @@
         <v>73</v>
       </c>
       <c r="B74" s="4" t="s">
-        <v>288</v>
+        <v>292</v>
       </c>
       <c r="C74" s="4" t="s">
-        <v>289</v>
+        <v>293</v>
       </c>
       <c r="D74" s="4" t="s">
-        <v>285</v>
+        <v>269</v>
       </c>
       <c r="E74" s="4" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
       <c r="F74" s="4" t="s">
-        <v>291</v>
+        <v>294</v>
       </c>
       <c r="G74" s="4" t="s">
         <v>20</v>
@@ -4965,19 +5109,19 @@
         <v>74</v>
       </c>
       <c r="B75" s="6" t="s">
-        <v>292</v>
+        <v>295</v>
       </c>
       <c r="C75" s="6" t="s">
-        <v>293</v>
+        <v>296</v>
       </c>
       <c r="D75" s="6" t="s">
-        <v>285</v>
+        <v>269</v>
       </c>
       <c r="E75" s="6" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="F75" s="6" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="G75" s="6" t="s">
         <v>20</v>
@@ -5012,19 +5156,19 @@
         <v>75</v>
       </c>
       <c r="B76" s="4" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="C76" s="4" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="D76" s="4" t="s">
-        <v>285</v>
+        <v>269</v>
       </c>
       <c r="E76" s="4" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="F76" s="4" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="G76" s="4" t="s">
         <v>20</v>
@@ -5059,13 +5203,13 @@
         <v>76</v>
       </c>
       <c r="B77" s="6" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="C77" s="6" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="D77" s="6" t="s">
-        <v>285</v>
+        <v>269</v>
       </c>
       <c r="E77" s="6" t="s">
         <v>302</v>
@@ -5112,13 +5256,13 @@
         <v>305</v>
       </c>
       <c r="D78" s="4" t="s">
-        <v>285</v>
+        <v>269</v>
       </c>
       <c r="E78" s="4" t="s">
+        <v>305</v>
+      </c>
+      <c r="F78" s="4" t="s">
         <v>306</v>
-      </c>
-      <c r="F78" s="4" t="s">
-        <v>307</v>
       </c>
       <c r="G78" s="4" t="s">
         <v>20</v>
@@ -5153,19 +5297,19 @@
         <v>78</v>
       </c>
       <c r="B79" s="6" t="s">
+        <v>307</v>
+      </c>
+      <c r="C79" s="6" t="s">
         <v>308</v>
       </c>
-      <c r="C79" s="6" t="s">
+      <c r="D79" s="6" t="s">
+        <v>269</v>
+      </c>
+      <c r="E79" s="6" t="s">
         <v>309</v>
       </c>
-      <c r="D79" s="6" t="s">
-        <v>285</v>
-      </c>
-      <c r="E79" s="6" t="s">
+      <c r="F79" s="6" t="s">
         <v>310</v>
-      </c>
-      <c r="F79" s="6" t="s">
-        <v>311</v>
       </c>
       <c r="G79" s="6" t="s">
         <v>20</v>
@@ -5200,19 +5344,19 @@
         <v>79</v>
       </c>
       <c r="B80" s="4" t="s">
+        <v>311</v>
+      </c>
+      <c r="C80" s="4" t="s">
         <v>312</v>
       </c>
-      <c r="C80" s="4" t="s">
+      <c r="D80" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="E80" s="4" t="s">
         <v>313</v>
       </c>
-      <c r="D80" s="4" t="s">
-        <v>285</v>
-      </c>
-      <c r="E80" s="4" t="s">
+      <c r="F80" s="4" t="s">
         <v>314</v>
-      </c>
-      <c r="F80" s="4" t="s">
-        <v>315</v>
       </c>
       <c r="G80" s="4" t="s">
         <v>20</v>
@@ -5247,19 +5391,19 @@
         <v>80</v>
       </c>
       <c r="B81" s="6" t="s">
+        <v>315</v>
+      </c>
+      <c r="C81" s="6" t="s">
         <v>316</v>
       </c>
-      <c r="C81" s="6" t="s">
+      <c r="D81" s="6" t="s">
+        <v>269</v>
+      </c>
+      <c r="E81" s="6" t="s">
         <v>317</v>
       </c>
-      <c r="D81" s="6" t="s">
-        <v>285</v>
-      </c>
-      <c r="E81" s="6" t="s">
+      <c r="F81" s="6" t="s">
         <v>318</v>
-      </c>
-      <c r="F81" s="6" t="s">
-        <v>319</v>
       </c>
       <c r="G81" s="6" t="s">
         <v>20</v>
@@ -5294,13 +5438,13 @@
         <v>81</v>
       </c>
       <c r="B82" s="4" t="s">
+        <v>319</v>
+      </c>
+      <c r="C82" s="4" t="s">
         <v>320</v>
       </c>
-      <c r="C82" s="4" t="s">
+      <c r="D82" s="4" t="s">
         <v>321</v>
-      </c>
-      <c r="D82" s="4" t="s">
-        <v>285</v>
       </c>
       <c r="E82" s="4" t="s">
         <v>322</v>
@@ -5347,7 +5491,7 @@
         <v>325</v>
       </c>
       <c r="D83" s="6" t="s">
-        <v>285</v>
+        <v>321</v>
       </c>
       <c r="E83" s="6" t="s">
         <v>326</v>
@@ -5394,7 +5538,7 @@
         <v>329</v>
       </c>
       <c r="D84" s="4" t="s">
-        <v>285</v>
+        <v>321</v>
       </c>
       <c r="E84" s="4" t="s">
         <v>330</v>
@@ -5441,7 +5585,7 @@
         <v>333</v>
       </c>
       <c r="D85" s="6" t="s">
-        <v>285</v>
+        <v>321</v>
       </c>
       <c r="E85" s="6" t="s">
         <v>334</v>
@@ -5488,7 +5632,7 @@
         <v>337</v>
       </c>
       <c r="D86" s="4" t="s">
-        <v>285</v>
+        <v>321</v>
       </c>
       <c r="E86" s="4" t="s">
         <v>338</v>
@@ -5524,19 +5668,583 @@
         <v>21</v>
       </c>
     </row>
+    <row r="87" spans="1:15" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A87" s="6">
+        <v>86</v>
+      </c>
+      <c r="B87" s="6" t="s">
+        <v>340</v>
+      </c>
+      <c r="C87" s="6" t="s">
+        <v>341</v>
+      </c>
+      <c r="D87" s="6" t="s">
+        <v>321</v>
+      </c>
+      <c r="E87" s="6" t="s">
+        <v>342</v>
+      </c>
+      <c r="F87" s="6" t="s">
+        <v>343</v>
+      </c>
+      <c r="G87" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="H87" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="I87" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="J87" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="K87" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="L87" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="M87" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="N87" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="O87" s="6" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="88" spans="1:15" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A88" s="4">
+        <v>87</v>
+      </c>
+      <c r="B88" s="4" t="s">
+        <v>344</v>
+      </c>
+      <c r="C88" s="4" t="s">
+        <v>345</v>
+      </c>
+      <c r="D88" s="4" t="s">
+        <v>321</v>
+      </c>
+      <c r="E88" s="4" t="s">
+        <v>346</v>
+      </c>
+      <c r="F88" s="4" t="s">
+        <v>347</v>
+      </c>
+      <c r="G88" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="H88" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="I88" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="J88" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="K88" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="L88" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="M88" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="N88" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="O88" s="4" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="89" spans="1:15" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A89" s="6">
+        <v>88</v>
+      </c>
+      <c r="B89" s="6" t="s">
+        <v>348</v>
+      </c>
+      <c r="C89" s="6" t="s">
+        <v>349</v>
+      </c>
+      <c r="D89" s="6" t="s">
+        <v>321</v>
+      </c>
+      <c r="E89" s="6" t="s">
+        <v>350</v>
+      </c>
+      <c r="F89" s="6" t="s">
+        <v>351</v>
+      </c>
+      <c r="G89" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="H89" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="I89" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="J89" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="K89" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="L89" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="M89" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="N89" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="O89" s="6" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="90" spans="1:15" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A90" s="4">
+        <v>89</v>
+      </c>
+      <c r="B90" s="4" t="s">
+        <v>352</v>
+      </c>
+      <c r="C90" s="4" t="s">
+        <v>353</v>
+      </c>
+      <c r="D90" s="4" t="s">
+        <v>321</v>
+      </c>
+      <c r="E90" s="4" t="s">
+        <v>354</v>
+      </c>
+      <c r="F90" s="4" t="s">
+        <v>355</v>
+      </c>
+      <c r="G90" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="H90" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="I90" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="J90" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="K90" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="L90" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="M90" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="N90" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="O90" s="4" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="91" spans="1:15" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A91" s="6">
+        <v>90</v>
+      </c>
+      <c r="B91" s="6" t="s">
+        <v>356</v>
+      </c>
+      <c r="C91" s="6" t="s">
+        <v>357</v>
+      </c>
+      <c r="D91" s="6" t="s">
+        <v>321</v>
+      </c>
+      <c r="E91" s="6" t="s">
+        <v>358</v>
+      </c>
+      <c r="F91" s="6" t="s">
+        <v>359</v>
+      </c>
+      <c r="G91" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="H91" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="I91" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="J91" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="K91" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="L91" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="M91" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="N91" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="O91" s="6" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="92" spans="1:15" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A92" s="4">
+        <v>91</v>
+      </c>
+      <c r="B92" s="4" t="s">
+        <v>360</v>
+      </c>
+      <c r="C92" s="4" t="s">
+        <v>361</v>
+      </c>
+      <c r="D92" s="4" t="s">
+        <v>321</v>
+      </c>
+      <c r="E92" s="4" t="s">
+        <v>362</v>
+      </c>
+      <c r="F92" s="4" t="s">
+        <v>363</v>
+      </c>
+      <c r="G92" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="H92" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="I92" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="J92" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="K92" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="L92" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="M92" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="N92" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="O92" s="4" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="93" spans="1:15" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A93" s="6">
+        <v>92</v>
+      </c>
+      <c r="B93" s="6" t="s">
+        <v>364</v>
+      </c>
+      <c r="C93" s="6" t="s">
+        <v>365</v>
+      </c>
+      <c r="D93" s="6" t="s">
+        <v>321</v>
+      </c>
+      <c r="E93" s="6" t="s">
+        <v>366</v>
+      </c>
+      <c r="F93" s="6" t="s">
+        <v>367</v>
+      </c>
+      <c r="G93" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="H93" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="I93" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="J93" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="K93" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="L93" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="M93" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="N93" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="O93" s="6" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="94" spans="1:15" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A94" s="4">
+        <v>93</v>
+      </c>
+      <c r="B94" s="4" t="s">
+        <v>368</v>
+      </c>
+      <c r="C94" s="4" t="s">
+        <v>369</v>
+      </c>
+      <c r="D94" s="4" t="s">
+        <v>321</v>
+      </c>
+      <c r="E94" s="4" t="s">
+        <v>370</v>
+      </c>
+      <c r="F94" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="G94" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="H94" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="I94" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="J94" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="K94" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="L94" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="M94" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="N94" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="O94" s="4" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="95" spans="1:15" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A95" s="6">
+        <v>94</v>
+      </c>
+      <c r="B95" s="6" t="s">
+        <v>372</v>
+      </c>
+      <c r="C95" s="6" t="s">
+        <v>373</v>
+      </c>
+      <c r="D95" s="6" t="s">
+        <v>321</v>
+      </c>
+      <c r="E95" s="6" t="s">
+        <v>374</v>
+      </c>
+      <c r="F95" s="6" t="s">
+        <v>375</v>
+      </c>
+      <c r="G95" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="H95" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="I95" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="J95" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="K95" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="L95" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="M95" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="N95" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="O95" s="6" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="96" spans="1:15" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A96" s="4">
+        <v>95</v>
+      </c>
+      <c r="B96" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="C96" s="4" t="s">
+        <v>377</v>
+      </c>
+      <c r="D96" s="4" t="s">
+        <v>321</v>
+      </c>
+      <c r="E96" s="4" t="s">
+        <v>378</v>
+      </c>
+      <c r="F96" s="4" t="s">
+        <v>379</v>
+      </c>
+      <c r="G96" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="H96" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="I96" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="J96" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="K96" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="L96" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="M96" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="N96" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="O96" s="4" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="97" spans="1:15" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A97" s="6">
+        <v>96</v>
+      </c>
+      <c r="B97" s="6" t="s">
+        <v>380</v>
+      </c>
+      <c r="C97" s="6" t="s">
+        <v>381</v>
+      </c>
+      <c r="D97" s="6" t="s">
+        <v>321</v>
+      </c>
+      <c r="E97" s="6" t="s">
+        <v>382</v>
+      </c>
+      <c r="F97" s="6" t="s">
+        <v>383</v>
+      </c>
+      <c r="G97" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="H97" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="I97" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="J97" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="K97" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="L97" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="M97" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="N97" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="O97" s="6" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="98" spans="1:15" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A98" s="4">
+        <v>97</v>
+      </c>
+      <c r="B98" s="4" t="s">
+        <v>384</v>
+      </c>
+      <c r="C98" s="4" t="s">
+        <v>385</v>
+      </c>
+      <c r="D98" s="4" t="s">
+        <v>321</v>
+      </c>
+      <c r="E98" s="4" t="s">
+        <v>386</v>
+      </c>
+      <c r="F98" s="4" t="s">
+        <v>387</v>
+      </c>
+      <c r="G98" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="H98" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="I98" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="J98" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="K98" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="L98" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="M98" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="N98" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="O98" s="4" t="s">
+        <v>21</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:O86"/>
+  <autoFilter ref="A1:O98"/>
   <dataValidations count="4">
-    <dataValidation type="list" allowBlank="1" sqref="H10:M86">
+    <dataValidation type="list" allowBlank="1" sqref="H10:M98">
       <formula1>"OK,NG,—"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="H2:M86">
+    <dataValidation type="list" allowBlank="1" sqref="H2:M98">
       <formula1>"OK,NG,—"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="N10:N86">
+    <dataValidation type="list" allowBlank="1" sqref="N10:N98">
       <formula1>"合格,要修正,未レビュー"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="N2:N86">
+    <dataValidation type="list" allowBlank="1" sqref="N2:N98">
       <formula1>"合格,要修正,未レビュー"</formula1>
     </dataValidation>
   </dataValidations>
@@ -5561,24 +6269,24 @@
         <v>3</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>340</v>
+        <v>388</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>341</v>
+        <v>389</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>342</v>
+        <v>390</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>343</v>
+        <v>391</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>69</v>
+        <v>77</v>
       </c>
       <c r="B2">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="C2">
         <v>0</v>
@@ -5592,7 +6300,7 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>233</v>
+        <v>269</v>
       </c>
       <c r="B3">
         <v>14</v>
@@ -5609,10 +6317,10 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>171</v>
+        <v>199</v>
       </c>
       <c r="B4">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -5626,10 +6334,10 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>285</v>
+        <v>321</v>
       </c>
       <c r="B5">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="C5">
         <v>0</v>
@@ -5646,7 +6354,7 @@
         <v>17</v>
       </c>
       <c r="B6">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="C6">
         <v>0</v>
@@ -5660,7 +6368,7 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>222</v>
+        <v>258</v>
       </c>
       <c r="B7">
         <v>3</v>
@@ -5677,7 +6385,7 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>123</v>
+        <v>151</v>
       </c>
       <c r="B8">
         <v>12</v>
@@ -5694,10 +6402,10 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>344</v>
+        <v>392</v>
       </c>
       <c r="B9">
-        <v>85</v>
+        <v>97</v>
       </c>
       <c r="C9">
         <v>0</v>

</xml_diff>